<commit_message>
docs: registrar fundação técnica e relatórios quinzenais 9 e 10
- adiciona decisão de reunião de 2026-10-01 (fundação técnica e equipe)
- atualiza DER v1, contexto, fluxos e funcionalidades da v1 mínima
- atualiza backlog completo, inventário e relatório de mudanças
- adiciona relatórios quinzenais 9 e 10 e relatório técnico do Ariel
</commit_message>
<xml_diff>
--- a/planejamento/backlog-completo.xlsx
+++ b/planejamento/backlog-completo.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista completa" sheetId="1" r:id="Rb008ebd89a8e412f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 9" sheetId="2" r:id="R11839390fbf0480b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 10" sheetId="3" r:id="R04e0006f8ffe49e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 11" sheetId="4" r:id="R25bf8dbc837e4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 12" sheetId="5" r:id="R7ed60e9680a44df1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 13" sheetId="6" r:id="R6509ce8ae4c7402b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 14" sheetId="7" r:id="Rdd2e41716f6f40dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista completa" sheetId="1" r:id="R49dfc9d0e28b482a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 9" sheetId="2" r:id="R8cc6ebbbd9cd4394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 10" sheetId="3" r:id="R3dcc78aacbb84a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 11" sheetId="4" r:id="R86ef82be84ba4dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 12" sheetId="5" r:id="R0768f0f3952c4d6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 13" sheetId="6" r:id="Rca5c7cef6aa640b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 14" sheetId="7" r:id="R100e86e044934e42"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -227,7 +227,7 @@
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
     <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Critério de aceite"/>
+    <x:tableColumn id="5" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -241,7 +241,7 @@
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
     <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Critério de aceite"/>
+    <x:tableColumn id="5" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -255,7 +255,7 @@
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
     <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Critério de aceite"/>
+    <x:tableColumn id="5" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -269,7 +269,7 @@
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
     <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Critério de aceite"/>
+    <x:tableColumn id="5" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -283,7 +283,7 @@
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
     <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Critério de aceite"/>
+    <x:tableColumn id="5" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -297,7 +297,7 @@
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
     <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Critério de aceite"/>
+    <x:tableColumn id="5" name="Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -504,7 +504,7 @@
     <x:col min="1" max="1" width="58" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -534,16 +534,16 @@
         <x:v>Descrição simples</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>Parecer Guilherme</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Observações</x:v>
+        <x:v>Integração/evidência</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
         <x:v>Tratamento do plano</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="28" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="19" t="str">
         <x:v>Consolidar fontes e decisões vigentes da V1</x:v>
       </x:c>
@@ -551,14 +551,16 @@
         <x:v>Reúne as fontes e decisões válidas que definem a V1.</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D5" s="19" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D5" s="19" t="str">
+        <x:v>Governança reconciliada neste snapshot de 12/10/2026.</x:v>
+      </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
         <x:v>Criar backlog normativo e planilha operacional por sprint</x:v>
       </x:c>
@@ -566,14 +568,16 @@
         <x:v>Cria o backlog oficial e uma planilha operacional organizada por sprint.</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D6" s="20" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="str">
+        <x:v>Governança reconciliada neste snapshot de 12/10/2026.</x:v>
+      </x:c>
       <x:c r="E6" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
         <x:v>Aplicar os três handoffs de 31/08 somente no snapshot</x:v>
       </x:c>
@@ -581,14 +585,16 @@
         <x:v>Aplica os três handoffs definidos em 31/08 somente no snapshot de design.</x:v>
       </x:c>
       <x:c r="C7" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D7" s="20" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D7" s="20" t="str">
+        <x:v>Protótipo entregue em agiliza-transparencia/origin/main (5a19a61).</x:v>
+      </x:c>
       <x:c r="E7" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
         <x:v>Validar visualmente os handoffs em 375, 768, 1024 e 1440 px</x:v>
       </x:c>
@@ -596,14 +602,16 @@
         <x:v>Confere visualmente os handoffs nos principais tamanhos de tela.</x:v>
       </x:c>
       <x:c r="C8" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D8" s="20" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D8" s="20" t="str">
+        <x:v>Protótipo entregue em agiliza-transparencia/origin/main (5a19a61).</x:v>
+      </x:c>
       <x:c r="E8" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="20" t="str">
         <x:v>Reconciliar o backlog com decisões e telas aprovadas</x:v>
       </x:c>
@@ -611,14 +619,16 @@
         <x:v>Compara o backlog com as decisões e telas já aprovadas.</x:v>
       </x:c>
       <x:c r="C9" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D9" s="20" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D9" s="20" t="str">
+        <x:v>Backlog e documentos derivados reconciliados neste snapshot de 12/10/2026.</x:v>
+      </x:c>
       <x:c r="E9" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="44" customHeight="1">
+    <x:row r="10" ht="48" hidden="0" customHeight="1">
       <x:c r="A10" s="24" t="str">
         <x:v>Inventariar e preparar a migração do ambiente local: interface, API, banco e ferramentas</x:v>
       </x:c>
@@ -626,14 +636,16 @@
         <x:v>Mapeia interface, API, banco e ferramentas para preparar a migração do ambiente local.</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D10" s="24" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="str">
+        <x:v>Inventário e preparação registrados no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E10" s="24" t="str">
         <x:v>Sprint 9</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="44" customHeight="1">
+    <x:row r="11" ht="72" hidden="0" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:v>Consolidar no repositório canônico guia, backlog, contratos-alvo e specs sanitizadas</x:v>
       </x:c>
@@ -641,14 +653,16 @@
         <x:v>Reúne guia, backlog, contratos e specs sanitizadas no repositório canônico.</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D11" s="24" t="str"/>
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="D11" s="24" t="str">
+        <x:v>Repositório canônico em main e memória técnica versionada.</x:v>
+      </x:c>
       <x:c r="E11" s="24" t="str">
         <x:v>Sprint 9</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="44" customHeight="1">
+    <x:row r="12" ht="60" hidden="0" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:v>Migrar seletivamente interface e API ao repositório canônico e ao único container de aplicação</x:v>
       </x:c>
@@ -656,14 +670,16 @@
         <x:v>Leva a interface e a API selecionadas para o repositório e container únicos.</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D12" s="24" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D12" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E12" s="24" t="str">
         <x:v>Sprint 9 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="44" customHeight="1">
+    <x:row r="13" ht="72" hidden="0" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:v>Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
@@ -671,14 +687,16 @@
         <x:v>Prepara a aplicação Laravel, o PostgreSQL externo e o desenvolvimento no container único.</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D13" s="24" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D13" s="24" t="str">
+        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+      </x:c>
       <x:c r="E13" s="24" t="str">
         <x:v>Sprint 9 e Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="44" customHeight="1">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="20" t="str">
         <x:v>Implementar health check, logs básicos e gate unificado de testes da aplicação</x:v>
       </x:c>
@@ -686,14 +704,16 @@
         <x:v>Cria a verificação de saúde, os registros básicos e uma etapa única de testes.</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D14" s="20" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D14" s="20" t="str">
+        <x:v>Gate de testes existe. Health check, logs básicos e correção do Compose continuam pendentes.</x:v>
+      </x:c>
       <x:c r="E14" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="44" customHeight="1">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="24" t="str">
         <x:v>Definir contexto de ator controlado e autorização desacoplada do login</x:v>
       </x:c>
@@ -701,14 +721,16 @@
         <x:v>Define quem está atuando e o que pode fazer sem depender diretamente do login.</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D15" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D15" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E15" s="24" t="str">
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="44" customHeight="1">
+    <x:row r="16" ht="60" hidden="0" customHeight="1">
       <x:c r="A16" s="24" t="str">
         <x:v>Aprovar e implementar o primeiro contrato HTTP real e cliente TypeScript</x:v>
       </x:c>
@@ -716,14 +738,16 @@
         <x:v>Implementa a primeira comunicação real entre frontend e backend com cliente TypeScript.</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D16" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D16" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E16" s="24" t="str">
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="44" customHeight="1">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="20" t="str">
         <x:v>Preparar fundação de homologação da aplicação em container único</x:v>
       </x:c>
@@ -731,14 +755,16 @@
         <x:v>Monta a base do ambiente de homologação usando o único container da aplicação.</x:v>
       </x:c>
       <x:c r="C17" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D17" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D17" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E17" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="44" customHeight="1">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="24" t="str">
         <x:v>Persistir o Catálogo mínimo e as UGs necessárias à publicação</x:v>
       </x:c>
@@ -746,14 +772,16 @@
         <x:v>Salva o catálogo mínimo e as unidades gestoras usadas para publicar ciclos.</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D18" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D18" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E18" s="24" t="str">
         <x:v>Sprint 11 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="44" customHeight="1">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="24" t="str">
         <x:v>Configurar ciclo de objeto variável sem modelo XLSX obrigatório</x:v>
       </x:c>
@@ -761,14 +789,16 @@
         <x:v>Permite configurar objeto variável sem exigir um modelo oficial de planilha.</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D19" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D19" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E19" s="24" t="str">
         <x:v>Sprint 11</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="44" customHeight="1">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="24" t="str">
         <x:v>Cadastrar e versionar modelo XLSX oficial obrigatório por objeto fixo</x:v>
       </x:c>
@@ -776,16 +806,16 @@
         <x:v>Cadastra e controla versões do modelo XLSX obrigatório de cada objeto fixo.</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>ok</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>só 1</x:v>
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
         <x:v>Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="44" customHeight="1">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="24" t="str">
         <x:v>Publicar ciclo de modo atômico e idempotente</x:v>
       </x:c>
@@ -793,14 +823,16 @@
         <x:v>Publica o ciclo por completo uma única vez, mesmo se houver repetição do comando.</x:v>
       </x:c>
       <x:c r="C21" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D21" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D21" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E21" s="24" t="str">
         <x:v>Sprint 11 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="44" customHeight="1">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="20" t="str">
         <x:v>Publicar sem SEI e congelar toggle focal por UG</x:v>
       </x:c>
@@ -808,14 +840,16 @@
         <x:v>Publica sem integração ao SEI e fixa a regra focal adequada para cada UG.</x:v>
       </x:c>
       <x:c r="C22" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D22" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D22" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E22" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="44" customHeight="1">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="24" t="str">
         <x:v>Integrar Criar Ciclo, Ciclos e Detalhe ao backend</x:v>
       </x:c>
@@ -823,14 +857,16 @@
         <x:v>Liga as telas de criação, lista e detalhe de ciclos ao backend real.</x:v>
       </x:c>
       <x:c r="C23" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D23" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D23" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E23" s="24" t="str">
         <x:v>Sprint 11 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="44" customHeight="1">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="20" t="str">
         <x:v>Auditar criação e publicação do ciclo</x:v>
       </x:c>
@@ -838,14 +874,16 @@
         <x:v>Registra em auditoria quem criou e publicou cada ciclo.</x:v>
       </x:c>
       <x:c r="C24" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D24" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D24" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E24" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="44" customHeight="1">
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="20" t="str">
         <x:v>Convidar respondentes e adjuntas por e-mail institucional</x:v>
       </x:c>
@@ -853,14 +891,16 @@
         <x:v>Envia convites a respondentes e adjuntas pelo e-mail institucional.</x:v>
       </x:c>
       <x:c r="C25" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D25" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D25" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E25" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="44" customHeight="1">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="24" t="str">
         <x:v>Criar atribuição e contribuição separada por pessoa e adjunta</x:v>
       </x:c>
@@ -868,14 +908,16 @@
         <x:v>Define a atribuição de cada pessoa e separa a contribuição da adjunta.</x:v>
       </x:c>
       <x:c r="C26" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D26" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D26" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E26" s="24" t="str">
         <x:v>Sprint 12</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="44" customHeight="1">
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="24" t="str">
         <x:v>Receber campos diretos e uploads em objeto variável sem modelo XLSX obrigatório</x:v>
       </x:c>
@@ -883,14 +925,16 @@
         <x:v>Recebe campos diretos e arquivos enviados para objeto variável, sem planilha oficial.</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D27" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D27" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E27" s="24" t="str">
         <x:v>Sprint 12</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="44" customHeight="1">
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="24" t="str">
         <x:v>Baixar, preencher e enviar o modelo XLSX oficial obrigatório do objeto fixo</x:v>
       </x:c>
@@ -898,14 +942,16 @@
         <x:v>Permite baixar, preencher e enviar o XLSX oficial exigido para objeto fixo.</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D28" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D28" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E28" s="24" t="str">
         <x:v>Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="44" customHeight="1">
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="24" t="str">
         <x:v>Salvar rascunho e arquivos vigentes em storage desacoplado</x:v>
       </x:c>
@@ -913,14 +959,16 @@
         <x:v>Guarda rascunhos e arquivos atuais em armazenamento separado da aplicação.</x:v>
       </x:c>
       <x:c r="C29" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D29" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D29" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E29" s="24" t="str">
         <x:v>Sprint 12 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="44" customHeight="1">
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="24" t="str">
         <x:v>Enviar pacote completo e emitir comprovante auditável</x:v>
       </x:c>
@@ -928,14 +976,16 @@
         <x:v>Envia a resposta completa e gera um comprovante que pode ser auditado.</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D30" s="24" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D30" s="24" t="str">
+        <x:v>Envio e download V1 estão implementados. O comprovante auditável permanece pendente.</x:v>
+      </x:c>
       <x:c r="E30" s="24" t="str">
         <x:v>Sprint 12 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="44" customHeight="1">
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="24" t="str">
         <x:v>Integrar painéis e contribuição às APIs da sprint</x:v>
       </x:c>
@@ -943,14 +993,16 @@
         <x:v>Conecta os painéis e a contribuição às APIs implementadas na sprint.</x:v>
       </x:c>
       <x:c r="C31" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D31" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D31" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E31" s="24" t="str">
         <x:v>Sprint 12 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="44" customHeight="1">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="20" t="str">
         <x:v>Aplicar modos direto, focal coordenador e focal observador</x:v>
       </x:c>
@@ -958,14 +1010,16 @@
         <x:v>Aplica os modos de resposta direta, focal coordenador e focal observador.</x:v>
       </x:c>
       <x:c r="C32" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D32" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D32" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E32" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="44" customHeight="1">
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="20" t="str">
         <x:v>Preservar o escopo durante a revisão focal</x:v>
       </x:c>
@@ -973,14 +1027,16 @@
         <x:v>Mantém o escopo definido enquanto a resposta passa pela revisão focal.</x:v>
       </x:c>
       <x:c r="C33" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D33" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D33" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E33" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="44" customHeight="1">
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="20" t="str">
         <x:v>Declarar ausência total de informações</x:v>
       </x:c>
@@ -988,14 +1044,16 @@
         <x:v>Permite informar formalmente que não há nenhuma informação a responder.</x:v>
       </x:c>
       <x:c r="C34" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D34" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D34" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E34" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="44" customHeight="1">
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="24" t="str">
         <x:v>Detectar campo direto ou upload ausente em objeto variável antes do envio</x:v>
       </x:c>
@@ -1003,14 +1061,16 @@
         <x:v>Bloqueia o envio de objeto variável quando não houver pelo menos um arquivo enviado.</x:v>
       </x:c>
       <x:c r="C35" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D35" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D35" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E35" s="24" t="str">
         <x:v>Sprint 11 e Sprint 12</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="44" customHeight="1">
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="24" t="str">
         <x:v>Validar o modelo XLSX obrigatório do objeto fixo antes do envio</x:v>
       </x:c>
@@ -1018,14 +1078,16 @@
         <x:v>Confere se o XLSX obrigatório do objeto fixo foi enviado corretamente.</x:v>
       </x:c>
       <x:c r="C36" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D36" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D36" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E36" s="24" t="str">
         <x:v>Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="44" customHeight="1">
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="20" t="str">
         <x:v>Confirmar não ocorrências e manter resposta parcial como respondida</x:v>
       </x:c>
@@ -1033,14 +1095,16 @@
         <x:v>Confirma não ocorrências e mantém uma resposta parcial como resposta válida.</x:v>
       </x:c>
       <x:c r="C37" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D37" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D37" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E37" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="44" customHeight="1">
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="20" t="str">
         <x:v>Conferir contribuições e encaminhar o conjunto focal à STC</x:v>
       </x:c>
@@ -1048,14 +1112,16 @@
         <x:v>Confere as contribuições e encaminha o conjunto focal para a STC.</x:v>
       </x:c>
       <x:c r="C38" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D38" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D38" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E38" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="44" customHeight="1">
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="20" t="str">
         <x:v>Apresentar pacote e completude para decisão humana da STC</x:v>
       </x:c>
@@ -1063,14 +1129,16 @@
         <x:v>Mostra o pacote e sua completude para a decisão humana da STC.</x:v>
       </x:c>
       <x:c r="C39" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D39" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D39" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E39" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="44" customHeight="1">
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="20" t="str">
         <x:v>Devolver contribuição ou item específico com um motivo</x:v>
       </x:c>
@@ -1078,14 +1146,16 @@
         <x:v>Devolve uma contribuição ou item específico, registrando o motivo.</x:v>
       </x:c>
       <x:c r="C40" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D40" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D40" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E40" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="44" customHeight="1">
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="20" t="str">
         <x:v>Corrigir e reenviar somente a contribuição afetada</x:v>
       </x:c>
@@ -1093,14 +1163,16 @@
         <x:v>Permite corrigir e reenviar apenas a contribuição que precisa de ajuste.</x:v>
       </x:c>
       <x:c r="C41" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D41" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D41" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E41" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="44" customHeight="1">
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="20" t="str">
         <x:v>Persistir o estado do ciclo, validar e permitir reversão controlada</x:v>
       </x:c>
@@ -1108,14 +1180,16 @@
         <x:v>Guarda o estado do ciclo, valida mudanças e permite reversão controlada.</x:v>
       </x:c>
       <x:c r="C42" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D42" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D42" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E42" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="44" customHeight="1">
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="20" t="str">
         <x:v>Separar auditoria de ciclo, coleta e respostas</x:v>
       </x:c>
@@ -1123,14 +1197,16 @@
         <x:v>Mantém auditorias separadas para ciclo, coleta e respostas.</x:v>
       </x:c>
       <x:c r="C43" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D43" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D43" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E43" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="44" customHeight="1">
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="20" t="str">
         <x:v>Integrar Validação e Histórico às APIs reais</x:v>
       </x:c>
@@ -1138,14 +1214,16 @@
         <x:v>Liga as telas de validação e histórico às APIs reais.</x:v>
       </x:c>
       <x:c r="C44" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D44" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D44" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E44" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="44" customHeight="1">
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="20" t="str">
         <x:v>Registrar números SEI e iniciar ou reiterar o prazo</x:v>
       </x:c>
@@ -1153,14 +1231,16 @@
         <x:v>Registra os números SEI e inicia ou repete o prazo do ciclo.</x:v>
       </x:c>
       <x:c r="C45" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D45" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D45" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E45" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="44" customHeight="1">
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="20" t="str">
         <x:v>Operar duas prorrogações separadas de cinco dias úteis</x:v>
       </x:c>
@@ -1168,14 +1248,16 @@
         <x:v>Controla duas prorrogações independentes de cinco dias úteis.</x:v>
       </x:c>
       <x:c r="C46" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D46" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D46" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E46" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="44" customHeight="1">
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="20" t="str">
         <x:v>Tratar solicitações de prorrogação pelo modo da UG</x:v>
       </x:c>
@@ -1183,14 +1265,16 @@
         <x:v>Trata pedidos de prorrogação conforme o modo de trabalho da UG.</x:v>
       </x:c>
       <x:c r="C47" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D47" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D47" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E47" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="44" customHeight="1">
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="20" t="str">
         <x:v>Encerrar manualmente coleta e ciclo</x:v>
       </x:c>
@@ -1198,14 +1282,16 @@
         <x:v>Permite encerrar manualmente a coleta e o ciclo quando necessário.</x:v>
       </x:c>
       <x:c r="C48" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D48" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D48" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E48" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="44" customHeight="1">
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="20" t="str">
         <x:v>Manter e exportar o Catálogo para ciclos futuros</x:v>
       </x:c>
@@ -1213,14 +1299,16 @@
         <x:v>Mantém e exporta o Catálogo para uso em ciclos futuros.</x:v>
       </x:c>
       <x:c r="C49" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D49" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D49" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E49" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="44" customHeight="1">
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="20" t="str">
         <x:v>Entregar dashboard operacional com unidades e drill-downs explícitos</x:v>
       </x:c>
@@ -1228,14 +1316,16 @@
         <x:v>Entrega painel operacional por unidade, com detalhamento acessível.</x:v>
       </x:c>
       <x:c r="C50" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D50" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D50" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E50" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="44" customHeight="1">
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="20" t="str">
         <x:v>Completar Histórico e consultas do Gabinete</x:v>
       </x:c>
@@ -1243,14 +1333,16 @@
         <x:v>Completa o histórico e as consultas disponíveis ao Gabinete.</x:v>
       </x:c>
       <x:c r="C51" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D51" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D51" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E51" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="44" customHeight="1">
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="20" t="str">
         <x:v>Copiar link e texto manual para uso no processo SEI</x:v>
       </x:c>
@@ -1258,14 +1350,16 @@
         <x:v>Gera link e texto para copiar manualmente no processo SEI.</x:v>
       </x:c>
       <x:c r="C52" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D52" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D52" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E52" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="44" customHeight="1">
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="20" t="str">
         <x:v>Operar o Diretório de UGs como consulta contextual</x:v>
       </x:c>
@@ -1273,14 +1367,16 @@
         <x:v>Disponibiliza o Diretório de UGs como consulta ligada ao contexto atual.</x:v>
       </x:c>
       <x:c r="C53" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D53" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D53" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E53" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="44" customHeight="1">
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="20" t="str">
         <x:v>Excluir ciclo sem apagar respostas armazenadas</x:v>
       </x:c>
@@ -1288,14 +1384,16 @@
         <x:v>Exclui o ciclo sem apagar as respostas que já foram armazenadas.</x:v>
       </x:c>
       <x:c r="C54" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D54" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D54" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E54" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="44" customHeight="1">
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="24" t="str">
         <x:v>Conectar login institucional ao contexto de ator</x:v>
       </x:c>
@@ -1303,14 +1401,16 @@
         <x:v>Relaciona o login institucional à pessoa que executará as ações no sistema.</x:v>
       </x:c>
       <x:c r="C55" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D55" s="24" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D55" s="24" t="str">
+        <x:v>Acesso V1 usa sessão local. Integração com login institucional permanece pendente.</x:v>
+      </x:c>
       <x:c r="E55" s="24" t="str">
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="44" customHeight="1">
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="24" t="str">
         <x:v>Conectar acesso contextual pelo link estável</x:v>
       </x:c>
@@ -1318,14 +1418,16 @@
         <x:v>Permite abrir o sistema pelo link estável já com o contexto correto de acesso.</x:v>
       </x:c>
       <x:c r="C56" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D56" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D56" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E56" s="24" t="str">
         <x:v>Sprint 11 e Sprint 12 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="44" customHeight="1">
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="24" t="str">
         <x:v>Aplicar isolamento definitivo de perfis, UGs e capacidades</x:v>
       </x:c>
@@ -1333,14 +1435,16 @@
         <x:v>Garante que cada perfil, UG e capacidade acesse somente o que lhe cabe.</x:v>
       </x:c>
       <x:c r="C57" s="24" t="str">
-        <x:v>ok</x:v>
-      </x:c>
-      <x:c r="D57" s="24" t="str"/>
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="D57" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
       <x:c r="E57" s="24" t="str">
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="44" customHeight="1">
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="20" t="str">
         <x:v>Exportar o filtro atual do Histórico em XLSX macro</x:v>
       </x:c>
@@ -1348,14 +1452,16 @@
         <x:v>Exporta em XLSX macro o filtro que estiver ativo no Histórico.</x:v>
       </x:c>
       <x:c r="C58" s="20" t="str">
-        <x:v>sem marcação</x:v>
-      </x:c>
-      <x:c r="D58" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D58" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E58" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="44" customHeight="1">
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="24" t="str">
         <x:v>Remover dados fictícios e acessos de demonstração do build de homologação</x:v>
       </x:c>
@@ -1363,14 +1469,16 @@
         <x:v>Remove dados e acessos de demonstração antes de usar o ambiente de homologação.</x:v>
       </x:c>
       <x:c r="C59" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D59" s="24" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D59" s="24" t="str">
+        <x:v>O caminho /v1 usa API real. Retirada dos dados demo para homologação permanece pendente.</x:v>
+      </x:c>
       <x:c r="E59" s="24" t="str">
         <x:v>Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="44" customHeight="1">
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="20" t="str">
         <x:v>Fechar segurança, upload, privacidade e retenção mínimas para o piloto</x:v>
       </x:c>
@@ -1378,14 +1486,16 @@
         <x:v>Fecha os requisitos mínimos de segurança, upload, privacidade e retenção para o piloto.</x:v>
       </x:c>
       <x:c r="C60" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D60" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D60" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E60" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="44" customHeight="1">
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="20" t="str">
         <x:v>Verificar observabilidade, backup, recuperação e rollback em homologação</x:v>
       </x:c>
@@ -1393,14 +1503,16 @@
         <x:v>Testa observabilidade, backup, recuperação e rollback no ambiente de homologação.</x:v>
       </x:c>
       <x:c r="C61" s="20" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D61" s="20" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D61" s="20" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E61" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="44" customHeight="1">
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="24" t="str">
         <x:v>Executar acessibilidade, responsividade, regressão e UAT ponta a ponta</x:v>
       </x:c>
@@ -1408,14 +1520,16 @@
         <x:v>Executa testes de acessibilidade, responsividade, regressão e UAT ponta a ponta.</x:v>
       </x:c>
       <x:c r="C62" s="24" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D62" s="24" t="str"/>
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="D62" s="24" t="str">
+        <x:v>Regressões automatizadas foram executadas. UAT e homologação ainda não ocorreram.</x:v>
+      </x:c>
       <x:c r="E62" s="24" t="str">
         <x:v>Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="44" customHeight="1">
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="21" t="str">
         <x:v>Emitir decisão de prontidão para piloto em homologação</x:v>
       </x:c>
@@ -1423,9 +1537,11 @@
         <x:v>Registra a decisão de que a aplicação está pronta, ou não, para o piloto em homologação.</x:v>
       </x:c>
       <x:c r="C63" s="21" t="str">
-        <x:v>nao</x:v>
-      </x:c>
-      <x:c r="D63" s="21" t="str"/>
+        <x:v>Planejado</x:v>
+      </x:c>
+      <x:c r="D63" s="21" t="str">
+        <x:v>Não iniciado no repositório canônico.</x:v>
+      </x:c>
       <x:c r="E63" s="25" t="str">
         <x:v>A definir</x:v>
       </x:c>
@@ -1433,7 +1549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde314bec34a141dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fe4c7061cf54ead"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1449,7 +1565,8 @@
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -1460,6 +1577,7 @@
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1469,6 +1587,11 @@
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -1481,13 +1604,16 @@
         <x:v>Atividade macro de origem</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Status</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Integração/evidência</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="64.5" customHeight="1">
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="19" t="str">
         <x:v>Inventariar código, banco e ferramentas</x:v>
       </x:c>
@@ -1498,13 +1624,16 @@
         <x:v>Inventariar e preparar a migração do ambiente local: interface, API, banco e ferramentas</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E5" s="19" t="str">
-        <x:v>Há um inventário seletivo sem documentos de contexto, e o fluxo e as regras do MVP estão preparados para revisão por PR.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="64.5" customHeight="1">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>Governança e inventário preparados para revisão técnica.</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
+        <x:v>Inventário, fluxo e regras foram preparados para revisão técnica.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
         <x:v>Preparar o repositório canônico</x:v>
       </x:c>
@@ -1515,13 +1644,16 @@
         <x:v>Consolidar no repositório canônico guia, backlog, contratos-alvo e specs sanitizadas | Migrar seletivamente interface e API ao repositório canônico e ao único container de aplicação</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str">
-        <x:v>O pacote de migração distingue código, specs sanitizadas e arquivos locais; nenhum documento bruto ou credencial é enviado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="64.5" customHeight="1">
+        <x:v>Concluído</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>Repositório canônico criado. Integração técnica segue em main e na branch V1.</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
+        <x:v>Repositório canônico criado; a migração seletiva do frontend foi implementada em fix-migracao e aguarda PR/merge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
         <x:v>Iniciar o container único</x:v>
       </x:c>
@@ -1532,13 +1664,16 @@
         <x:v>Inventariar e preparar a migração do ambiente local: interface, API, banco e ferramentas | Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
       <x:c r="D7" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E7" s="20" t="str">
-        <x:v>Existe uma estrutura inicial do container da aplicação e a comunicação com um PostgreSQL separado está prevista para completar na Sprint 10.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="82.5" customHeight="1">
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="str">
+        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
+        <x:v>Não há container de aplicação configurado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="21" t="str">
         <x:v>Iniciar Laravel e a conexão PostgreSQL</x:v>
       </x:c>
@@ -1549,13 +1684,16 @@
         <x:v>Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E8" s="21" t="str">
-        <x:v>A fundação de Guilherme inicia sem segredo versionado; a conexão local usa o PostgreSQL separado e pode ser trocada por configuração quando os parâmetros forem fornecidos.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="105" customHeight="1">
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="E8" s="31" t="str">
+        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+      </x:c>
+      <x:c r="F8" s="21" t="str">
+        <x:v>Laravel/Inertia existe; PostgreSQL externo ainda não foi configurado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="35" t="str">
         <x:v>Preparar fluxo e regras do backend</x:v>
       </x:c>
@@ -1566,16 +1704,19 @@
         <x:v>Definir o fluxo principal de coleta, resposta, validação e entrega da V1</x:v>
       </x:c>
       <x:c r="D9" s="35" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="35" t="str">
-        <x:v>Há uma matriz local de regras e testes de contrato propostos, sem inventar endpoints ou credenciais.</x:v>
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F9" s="35" t="str">
+        <x:v>Fluxo V1, regras e handoff técnico documentados; contrato HTTP continua pendente.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R009c2a7a55674ac2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d439cdaa1e24184"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1591,7 +1732,8 @@
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -1602,6 +1744,7 @@
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1611,6 +1754,11 @@
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -1623,13 +1771,16 @@
         <x:v>Atividade macro de origem</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Status</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Integração/evidência</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="44" customHeight="1">
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="19" t="str">
         <x:v>Concluir a fundação Laravel e PostgreSQL</x:v>
       </x:c>
@@ -1640,13 +1791,16 @@
         <x:v>Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E5" s="19" t="str">
-        <x:v>A aplicação persiste dados básicos no PostgreSQL externo.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
+        <x:v>Laravel/Inertia iniciado; PostgreSQL externo bloqueado até alinhamento técnico com a STC.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="20" t="str">
         <x:v>Criar o primeiro endpoint HTTP</x:v>
       </x:c>
@@ -1657,13 +1811,16 @@
         <x:v>Aprovar e implementar o primeiro contrato HTTP real e cliente TypeScript</x:v>
       </x:c>
       <x:c r="D6" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str">
-        <x:v>Uma rota retorna dados reais do backend.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E6" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
+        <x:v>Aguardar contrato de dados, infraestrutura e estratégia de homologação definidos com a STC.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="20" t="str">
         <x:v>Conectar a primeira tela à API</x:v>
       </x:c>
@@ -1674,13 +1831,16 @@
         <x:v>Aprovar e implementar o primeiro contrato HTTP real e cliente TypeScript</x:v>
       </x:c>
       <x:c r="D7" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E7" s="20" t="str">
-        <x:v>A tela recebe dados pelo caminho /api sem fixture como fonte operacional.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="76" customHeight="1">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
+        <x:v>Depende do primeiro contrato HTTP aprovado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" hidden="0" customHeight="1">
       <x:c r="A8" s="20" t="str">
         <x:v>Criar grupos Administrador/STC e Respondente</x:v>
       </x:c>
@@ -1691,13 +1851,16 @@
         <x:v>Definir contexto de ator controlado e autorização desacoplada do login | Conectar login institucional ao contexto de ator | Aplicar isolamento definitivo de perfis, UGs e capacidades</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E8" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
         <x:v>Administrador/STC e Respondente possuem ações diferentes no MVP.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="60" customHeight="1">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="21" t="str">
         <x:v>Vincular usuários a UGs e grupos</x:v>
       </x:c>
@@ -1708,16 +1871,19 @@
         <x:v>Definir contexto de ator controlado e autorização desacoplada do login | Aplicar isolamento definitivo de perfis, UGs e capacidades</x:v>
       </x:c>
       <x:c r="D9" s="32" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E9" s="21" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E9" s="32" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F9" s="21" t="str">
         <x:v>Respondente não visualiza pedido de outra UG.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2585f55e26fa4188"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45bd9841c1144610"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1733,7 +1899,8 @@
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -1744,6 +1911,7 @@
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1753,6 +1921,11 @@
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -1765,9 +1938,12 @@
         <x:v>Atividade macro de origem</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Status</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Integração/evidência</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
@@ -1782,9 +1958,12 @@
         <x:v>Persistir o Catálogo mínimo e as UGs necessárias à publicação</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E5" s="19" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E5" s="27" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
         <x:v>STC seleciona um objeto variável e uma UG.</x:v>
       </x:c>
     </x:row>
@@ -1799,9 +1978,12 @@
         <x:v>Configurar ciclo de objeto variável sem modelo XLSX obrigatório</x:v>
       </x:c>
       <x:c r="D6" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E6" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
         <x:v>STC cria uma coleta variável com objeto, UG e item solicitado.</x:v>
       </x:c>
     </x:row>
@@ -1816,9 +1998,12 @@
         <x:v>Configurar ciclo de objeto variável sem modelo XLSX obrigatório | Detectar campo direto ou upload ausente em objeto variável antes do envio</x:v>
       </x:c>
       <x:c r="D7" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E7" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
         <x:v>A coleta variável deixa explícita a exigência de upload.</x:v>
       </x:c>
     </x:row>
@@ -1833,9 +2018,12 @@
         <x:v>Publicar ciclo de modo atômico e idempotente</x:v>
       </x:c>
       <x:c r="D8" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E8" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E8" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
         <x:v>A publicação cria uma coleta sem estado parcial.</x:v>
       </x:c>
     </x:row>
@@ -1850,9 +2038,12 @@
         <x:v>Publicar ciclo de modo atômico e idempotente | Conectar acesso contextual pelo link estável</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E9" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
         <x:v>Abrir o link leva ao pedido correspondente.</x:v>
       </x:c>
     </x:row>
@@ -1867,16 +2058,19 @@
         <x:v>Integrar Criar Ciclo, Ciclos e Detalhe ao backend</x:v>
       </x:c>
       <x:c r="D10" s="32" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E10" s="21" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E10" s="32" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F10" s="21" t="str">
         <x:v>STC cria, publica e consulta a coleta variável sem ciclo demonstrativo.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52ac6977345f4a5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3544fced55348a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1892,7 +2086,8 @@
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -1903,6 +2098,7 @@
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -1912,6 +2108,11 @@
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -1924,9 +2125,12 @@
         <x:v>Atividade macro de origem</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Status</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Integração/evidência</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
@@ -1941,9 +2145,12 @@
         <x:v>Conectar acesso contextual pelo link estável</x:v>
       </x:c>
       <x:c r="D5" s="33" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E5" s="19" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E5" s="33" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
         <x:v>O link não mostra pedidos de outras UGs.</x:v>
       </x:c>
     </x:row>
@@ -1958,9 +2165,12 @@
         <x:v>Criar atribuição e contribuição separada por pessoa e adjunta | Conectar acesso contextual pelo link estável</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
         <x:v>O respondente entra na contribuição correta sem SSO institucional completo.</x:v>
       </x:c>
     </x:row>
@@ -1975,9 +2185,12 @@
         <x:v>Receber campos diretos e uploads em objeto variável sem modelo XLSX obrigatório</x:v>
       </x:c>
       <x:c r="D7" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E7" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
         <x:v>O respondente visualiza os itens solicitados.</x:v>
       </x:c>
     </x:row>
@@ -1992,9 +2205,12 @@
         <x:v>Receber campos diretos e uploads em objeto variável sem modelo XLSX obrigatório | Salvar rascunho e arquivos vigentes em storage desacoplado</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E8" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
         <x:v>O arquivo permanece disponível até o envio da resposta.</x:v>
       </x:c>
     </x:row>
@@ -2009,9 +2225,12 @@
         <x:v>Detectar campo direto ou upload ausente em objeto variável antes do envio</x:v>
       </x:c>
       <x:c r="D9" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E9" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E9" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
         <x:v>O sistema bloqueia o envio quando não existe upload.</x:v>
       </x:c>
     </x:row>
@@ -2026,9 +2245,12 @@
         <x:v>Enviar pacote completo e emitir comprovante auditável</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E10" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E10" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F10" s="20" t="str">
         <x:v>A resposta sai do respondente e fica disponível para a STC.</x:v>
       </x:c>
     </x:row>
@@ -2043,16 +2265,19 @@
         <x:v>Integrar painéis e contribuição às APIs da sprint</x:v>
       </x:c>
       <x:c r="D11" s="32" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E11" s="21" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E11" s="32" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F11" s="21" t="str">
         <x:v>STC localiza a resposta variável e baixa seu arquivo.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f6377d0ca4f4108"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76a4fac573c44af1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2068,7 +2293,8 @@
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -2079,6 +2305,7 @@
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -2088,6 +2315,11 @@
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -2100,9 +2332,12 @@
         <x:v>Atividade macro de origem</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Status</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Integração/evidência</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
@@ -2117,9 +2352,12 @@
         <x:v>Persistir o Catálogo mínimo e as UGs necessárias à publicação | Cadastrar e versionar modelo XLSX oficial obrigatório por objeto fixo</x:v>
       </x:c>
       <x:c r="D5" s="33" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E5" s="19" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E5" s="33" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
         <x:v>Existe um objeto fixo disponível para criar uma coleta.</x:v>
       </x:c>
     </x:row>
@@ -2134,9 +2372,12 @@
         <x:v>Cadastrar e versionar modelo XLSX oficial obrigatório por objeto fixo</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
         <x:v>O objeto fixo possui um modelo XLSX disponível.</x:v>
       </x:c>
     </x:row>
@@ -2151,9 +2392,12 @@
         <x:v>Publicar ciclo de modo atômico e idempotente | Conectar acesso contextual pelo link estável</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E7" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
         <x:v>A coleta fixa tem link próprio e referência ao modelo.</x:v>
       </x:c>
     </x:row>
@@ -2168,9 +2412,12 @@
         <x:v>Baixar, preencher e enviar o modelo XLSX oficial obrigatório do objeto fixo</x:v>
       </x:c>
       <x:c r="D8" s="29" t="str">
-        <x:v>Planejado</x:v>
-      </x:c>
-      <x:c r="E8" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E8" s="29" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
         <x:v>O respondente baixa o XLSX vinculado à coleta fixa.</x:v>
       </x:c>
     </x:row>
@@ -2185,9 +2432,12 @@
         <x:v>Baixar, preencher e enviar o modelo XLSX oficial obrigatório do objeto fixo | Salvar rascunho e arquivos vigentes em storage desacoplado</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E9" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E9" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F9" s="20" t="str">
         <x:v>O respondente envia a planilha preenchida como arquivo principal.</x:v>
       </x:c>
     </x:row>
@@ -2202,16 +2452,19 @@
         <x:v>Validar o modelo XLSX obrigatório do objeto fixo antes do envio</x:v>
       </x:c>
       <x:c r="D10" s="32" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E10" s="21" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E10" s="32" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F10" s="21" t="str">
         <x:v>Arquivo incompatível é recusado e o modelo correto segue para envio.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3656f68f7b564b1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f20e08f00ee4dd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2227,7 +2480,8 @@
     <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="46" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
@@ -2238,6 +2492,7 @@
       <x:c r="C1" s="3"/>
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
+      <x:c r="F1" s="3"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -2247,6 +2502,11 @@
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
       <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="E3"/>
+      <x:c r="F3"/>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -2259,9 +2519,12 @@
         <x:v>Atividade macro de origem</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Status</x:v>
+        <x:v>Status técnico</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
+        <x:v>Integração/evidência</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
@@ -2276,9 +2539,12 @@
         <x:v>Enviar pacote completo e emitir comprovante auditável</x:v>
       </x:c>
       <x:c r="D5" s="33" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E5" s="19" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E5" s="33" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F5" s="19" t="str">
         <x:v>A resposta fixa fica disponível para a STC.</x:v>
       </x:c>
     </x:row>
@@ -2293,9 +2559,12 @@
         <x:v>Integrar painéis e contribuição às APIs da sprint</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str">
+        <x:v>Concluído tecnicamente</x:v>
+      </x:c>
+      <x:c r="E6" s="24" t="str">
+        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+      </x:c>
+      <x:c r="F6" s="20" t="str">
         <x:v>STC localiza e baixa a planilha oficial.</x:v>
       </x:c>
     </x:row>
@@ -2310,9 +2579,12 @@
         <x:v>Migrar seletivamente interface e API ao repositório canônico e ao único container de aplicação | Integrar Criar Ciclo, Ciclos e Detalhe ao backend | Integrar painéis e contribuição às APIs da sprint | Remover dados fictícios e acessos de demonstração do build de homologação</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E7" s="20" t="str">
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="E7" s="24" t="str">
+        <x:v>O caminho /v1 usa API real. Retirada dos dados demo para homologação permanece pendente.</x:v>
+      </x:c>
+      <x:c r="F7" s="20" t="str">
         <x:v>O caminho variável não depende de dados demonstrativos.</x:v>
       </x:c>
     </x:row>
@@ -2327,9 +2599,12 @@
         <x:v>Migrar seletivamente interface e API ao repositório canônico e ao único container de aplicação | Integrar Criar Ciclo, Ciclos e Detalhe ao backend | Integrar painéis e contribuição às APIs da sprint | Remover dados fictícios e acessos de demonstração do build de homologação</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E8" s="20" t="str">
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="E8" s="24" t="str">
+        <x:v>O caminho /v1 usa API real. Retirada dos dados demo para homologação permanece pendente.</x:v>
+      </x:c>
+      <x:c r="F8" s="20" t="str">
         <x:v>O caminho fixo não depende de dados demonstrativos.</x:v>
       </x:c>
     </x:row>
@@ -2344,16 +2619,19 @@
         <x:v>Executar acessibilidade, responsividade, regressão e UAT ponta a ponta</x:v>
       </x:c>
       <x:c r="D9" s="32" t="str">
-        <x:v>Recorte</x:v>
-      </x:c>
-      <x:c r="E9" s="21" t="str">
+        <x:v>Em andamento</x:v>
+      </x:c>
+      <x:c r="E9" s="32" t="str">
+        <x:v>Regressões automatizadas passaram. O build da imagem app do Compose ainda bloqueia o fechamento.</x:v>
+      </x:c>
+      <x:c r="F9" s="21" t="str">
         <x:v>Não há defeito bloqueante nos dois fluxos mínimos.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18dbb79e9bf74d53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a684c4003144579"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: registrar merge do PR 5
</commit_message>
<xml_diff>
--- a/planejamento/backlog-completo.xlsx
+++ b/planejamento/backlog-completo.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista completa" sheetId="1" r:id="R49dfc9d0e28b482a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 9" sheetId="2" r:id="R8cc6ebbbd9cd4394"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 10" sheetId="3" r:id="R3dcc78aacbb84a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 11" sheetId="4" r:id="R86ef82be84ba4dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 12" sheetId="5" r:id="R0768f0f3952c4d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 13" sheetId="6" r:id="Rca5c7cef6aa640b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 14" sheetId="7" r:id="R100e86e044934e42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista completa" sheetId="1" r:id="Ra87d11e30882435f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 9" sheetId="2" r:id="Rf8e918af6bd54649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 10" sheetId="3" r:id="Rea456881755c45a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 11" sheetId="4" r:id="R5ee7e4de180b4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 12" sheetId="5" r:id="R2abbcaf0e75f4afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 13" sheetId="6" r:id="Re74f45f402244ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 14" sheetId="7" r:id="Ra62832aa173c485d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -673,7 +673,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E12" s="24" t="str">
         <x:v>Sprint 9 e Sprint 14</x:v>
@@ -690,7 +690,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
       </x:c>
       <x:c r="E13" s="24" t="str">
         <x:v>Sprint 9 e Sprint 10</x:v>
@@ -704,10 +704,10 @@
         <x:v>Cria a verificação de saúde, os registros básicos e uma etapa única de testes.</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D14" s="20" t="str">
-        <x:v>Gate de testes existe. Health check, logs básicos e correção do Compose continuam pendentes.</x:v>
+        <x:v>Health check /up, logs em stderr e composer ci:check existem; docker compose build app verificado em 14/10/2026.</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
         <x:v>A definir</x:v>
@@ -724,7 +724,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
         <x:v>Sprint 10</x:v>
@@ -741,7 +741,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E16" s="24" t="str">
         <x:v>Sprint 10</x:v>
@@ -775,7 +775,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
         <x:v>Sprint 11 e Sprint 13</x:v>
@@ -792,7 +792,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
         <x:v>Sprint 11</x:v>
@@ -809,7 +809,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
         <x:v>Sprint 13</x:v>
@@ -826,7 +826,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D21" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E21" s="24" t="str">
         <x:v>Sprint 11 e Sprint 13</x:v>
@@ -860,7 +860,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D23" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E23" s="24" t="str">
         <x:v>Sprint 11 e Sprint 14</x:v>
@@ -911,7 +911,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
         <x:v>Sprint 12</x:v>
@@ -928,7 +928,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
         <x:v>Sprint 12</x:v>
@@ -945,7 +945,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E28" s="24" t="str">
         <x:v>Sprint 13</x:v>
@@ -962,7 +962,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D29" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E29" s="24" t="str">
         <x:v>Sprint 12 e Sprint 13</x:v>
@@ -996,7 +996,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D31" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E31" s="24" t="str">
         <x:v>Sprint 12 e Sprint 14</x:v>
@@ -1064,7 +1064,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D35" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E35" s="24" t="str">
         <x:v>Sprint 11 e Sprint 12</x:v>
@@ -1081,7 +1081,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D36" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E36" s="24" t="str">
         <x:v>Sprint 13</x:v>
@@ -1421,7 +1421,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D56" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E56" s="24" t="str">
         <x:v>Sprint 11 e Sprint 12 e Sprint 13</x:v>
@@ -1438,7 +1438,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D57" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="E57" s="24" t="str">
         <x:v>Sprint 10</x:v>
@@ -1549,7 +1549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8fe4c7061cf54ead"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ce700d608074e2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1667,7 +1667,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>Não há container de aplicação configurado.</x:v>
@@ -1687,7 +1687,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E8" s="31" t="str">
-        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
       </x:c>
       <x:c r="F8" s="21" t="str">
         <x:v>Laravel/Inertia existe; PostgreSQL externo ainda não foi configurado.</x:v>
@@ -1707,7 +1707,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="35" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F9" s="35" t="str">
         <x:v>Fluxo V1, regras e handoff técnico documentados; contrato HTTP continua pendente.</x:v>
@@ -1716,7 +1716,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d439cdaa1e24184"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02cd1a5700b24d46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1794,7 +1794,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Base em main (ecb6c05). PostgreSQL e migrations foram validados, mas o build da imagem app do Compose falha.</x:v>
+        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>Laravel/Inertia iniciado; PostgreSQL externo bloqueado até alinhamento técnico com a STC.</x:v>
@@ -1814,7 +1814,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E6" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>Aguardar contrato de dados, infraestrutura e estratégia de homologação definidos com a STC.</x:v>
@@ -1834,7 +1834,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>Depende do primeiro contrato HTTP aprovado.</x:v>
@@ -1854,7 +1854,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:v>Administrador/STC e Respondente possuem ações diferentes no MVP.</x:v>
@@ -1874,7 +1874,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
         <x:v>Respondente não visualiza pedido de outra UG.</x:v>
@@ -1883,7 +1883,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45bd9841c1144610"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d7291a4f1b24db1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1961,7 +1961,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>STC seleciona um objeto variável e uma UG.</x:v>
@@ -1981,7 +1981,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E6" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>STC cria uma coleta variável com objeto, UG e item solicitado.</x:v>
@@ -2001,7 +2001,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>A coleta variável deixa explícita a exigência de upload.</x:v>
@@ -2021,7 +2021,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E8" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:v>A publicação cria uma coleta sem estado parcial.</x:v>
@@ -2041,7 +2041,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>Abrir o link leva ao pedido correspondente.</x:v>
@@ -2061,7 +2061,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E10" s="32" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F10" s="21" t="str">
         <x:v>STC cria, publica e consulta a coleta variável sem ciclo demonstrativo.</x:v>
@@ -2070,7 +2070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3544fced55348a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R807740a09a334e54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2148,7 +2148,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>O link não mostra pedidos de outras UGs.</x:v>
@@ -2168,7 +2168,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>O respondente entra na contribuição correta sem SSO institucional completo.</x:v>
@@ -2188,7 +2188,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>O respondente visualiza os itens solicitados.</x:v>
@@ -2208,7 +2208,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:v>O arquivo permanece disponível até o envio da resposta.</x:v>
@@ -2228,7 +2228,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>O sistema bloqueia o envio quando não existe upload.</x:v>
@@ -2248,7 +2248,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E10" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
         <x:v>A resposta sai do respondente e fica disponível para a STC.</x:v>
@@ -2268,7 +2268,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E11" s="32" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F11" s="21" t="str">
         <x:v>STC localiza a resposta variável e baixa seu arquivo.</x:v>
@@ -2277,7 +2277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76a4fac573c44af1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99f9af4a6b1f4826"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2355,7 +2355,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>Existe um objeto fixo disponível para criar uma coleta.</x:v>
@@ -2375,7 +2375,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>O objeto fixo possui um modelo XLSX disponível.</x:v>
@@ -2395,7 +2395,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>A coleta fixa tem link próprio e referência ao modelo.</x:v>
@@ -2415,7 +2415,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E8" s="29" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:v>O respondente baixa o XLSX vinculado à coleta fixa.</x:v>
@@ -2435,7 +2435,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>O respondente envia a planilha preenchida como arquivo principal.</x:v>
@@ -2455,7 +2455,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E10" s="32" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F10" s="21" t="str">
         <x:v>Arquivo incompatível é recusado e o modelo correto segue para envio.</x:v>
@@ -2464,7 +2464,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f20e08f00ee4dd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb30e8e7210bc4038"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2542,7 +2542,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>A resposta fixa fica disponível para a STC.</x:v>
@@ -2562,7 +2562,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>Implementado em origin/fluxos-http-v1 (0d2d832), 9 commits à frente de origin/main. Integração em main pendente.</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>STC localiza e baixa a planilha oficial.</x:v>
@@ -2622,7 +2622,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
-        <x:v>Regressões automatizadas passaram. O build da imagem app do Compose ainda bloqueia o fechamento.</x:v>
+        <x:v>Regressões automatizadas e docker compose build app passaram. UAT e homologação continuam pendentes.</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
         <x:v>Não há defeito bloqueante nos dois fluxos mínimos.</x:v>
@@ -2631,7 +2631,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a684c4003144579"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc60319396364ee8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(governanca): atualizar governança até o PR #12
- v1-minima, rastreabilidade, contexto, regras de negócio (8.2) e DER
  registram o comprovante em PDF (PR #10) e a preparação para
  homologação (PR #11)
- fluxos V1 e handoff do backend refletem a revisão de 17/10, com SVGs
  regerados
- contexto §28 lista as pendências de implantação da V1
- backlog com status e evidências atualizados
- Tesauro v2.3 retirado do acervo, substituído pela v2.6
- relatório síntese de outubro incluído no inventário
</commit_message>
<xml_diff>
--- a/planejamento/backlog-completo.xlsx
+++ b/planejamento/backlog-completo.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista completa" sheetId="1" r:id="Ra87d11e30882435f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 9" sheetId="2" r:id="Rf8e918af6bd54649"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 10" sheetId="3" r:id="Rea456881755c45a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 11" sheetId="4" r:id="R5ee7e4de180b4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 12" sheetId="5" r:id="R2abbcaf0e75f4afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 13" sheetId="6" r:id="Re74f45f402244ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 14" sheetId="7" r:id="Ra62832aa173c485d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista completa" sheetId="1" r:id="R9dbf21a979d24d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 9" sheetId="2" r:id="Rf9e0b6c18fb848fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 10" sheetId="3" r:id="R1cfe3389b09a41cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 11" sheetId="4" r:id="Rd38b1b60d9074e2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 12" sheetId="5" r:id="R2134b194f94c4464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 13" sheetId="6" r:id="R2bf75d68130b4640"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 14" sheetId="7" r:id="R889c2377c7f84121"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -696,7 +696,7 @@
         <x:v>Sprint 9 e Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
       <x:c r="A14" s="20" t="str">
         <x:v>Implementar health check, logs básicos e gate unificado de testes da aplicação</x:v>
       </x:c>
@@ -704,10 +704,10 @@
         <x:v>Cria a verificação de saúde, os registros básicos e uma etapa única de testes.</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
-        <x:v>Concluído tecnicamente</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D14" s="20" t="str">
-        <x:v>Health check /up, logs em stderr e composer ci:check existem; docker compose build app verificado em 14/10/2026.</x:v>
+        <x:v>Health check /up, logs em stderr e composer ci:check existem em main. O GitHub está sem CI desde 05/10/2026 (6ac78e3); a evidência é a bateria local registrada no repositório canônico.</x:v>
       </x:c>
       <x:c r="E14" s="23" t="str">
         <x:v>A definir</x:v>
@@ -755,10 +755,10 @@
         <x:v>Monta a base do ambiente de homologação usando o único container da aplicação.</x:v>
       </x:c>
       <x:c r="C17" s="20" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D17" s="20" t="str">
-        <x:v>Não iniciado no repositório canônico.</x:v>
+        <x:v>Imagem de produção ensaiada atrás de proxy HTTPS, com guia do ambiente e roteiro de UAT, em main (18c345b, PR #11 mesclado em 19/10/2026). Ambiente real e hospedagem pendentes.</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
         <x:v>A definir</x:v>
@@ -928,7 +928,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 17/10/2026 a resposta é só por arquivos, sem campos diretos (main 18c345b).</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
         <x:v>Sprint 12</x:v>
@@ -962,7 +962,7 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D29" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 17/10/2026 o arquivo fica guardado ao ser escolhido, sem botão Salvar rascunho (main 18c345b).</x:v>
       </x:c>
       <x:c r="E29" s="24" t="str">
         <x:v>Sprint 12 e Sprint 13</x:v>
@@ -976,10 +976,10 @@
         <x:v>Envia a resposta completa e gera um comprovante que pode ser auditado.</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
-        <x:v>Envio e download V1 estão implementados. O comprovante auditável permanece pendente.</x:v>
+        <x:v>Envio auditável e comprovante PDF em main (849c522, PR #10 mesclado em 16/10/2026). Reenvio e adjuntas dependem de fluxos futuros.</x:v>
       </x:c>
       <x:c r="E30" s="24" t="str">
         <x:v>Sprint 12 e Sprint 14</x:v>
@@ -1404,7 +1404,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D55" s="24" t="str">
-        <x:v>Acesso V1 usa sessão local. Integração com login institucional permanece pendente.</x:v>
+        <x:v>Acesso V1 usa sessão local; contas STC são criadas por comando (stc:create-user, main 18c345b). Login institucional e processo de contas STC pendentes.</x:v>
       </x:c>
       <x:c r="E55" s="24" t="str">
         <x:v>Sprint 10</x:v>
@@ -1472,7 +1472,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D59" s="24" t="str">
-        <x:v>O caminho /v1 usa API real. Retirada dos dados demo para homologação permanece pendente.</x:v>
+        <x:v>Em produção a imagem serve só a V1, sem as telas do protótipo (main 18c345b). Carga do piloto preparada, mas não executada em base operacional. A demo com dados fictícios fica só no Render (deploy/demo-render).</x:v>
       </x:c>
       <x:c r="E59" s="24" t="str">
         <x:v>Sprint 14</x:v>
@@ -1486,10 +1486,10 @@
         <x:v>Fecha os requisitos mínimos de segurança, upload, privacidade e retenção para o piloto.</x:v>
       </x:c>
       <x:c r="C60" s="20" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D60" s="20" t="str">
-        <x:v>Não iniciado no repositório canônico.</x:v>
+        <x:v>Arquivos em disco privado com download autorizado, teto de 10 MiB e 20 arquivos por resposta, tentativas limitadas por rota e cabeçalhos de segurança em main (18c345b). Varredura de arquivos e retenção pendentes.</x:v>
       </x:c>
       <x:c r="E60" s="23" t="str">
         <x:v>A definir</x:v>
@@ -1503,10 +1503,10 @@
         <x:v>Testa observabilidade, backup, recuperação e rollback no ambiente de homologação.</x:v>
       </x:c>
       <x:c r="C61" s="20" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D61" s="20" t="str">
-        <x:v>Não iniciado no repositório canônico.</x:v>
+        <x:v>Cópia e restauração conjunta de banco e arquivos ensaiadas no roteiro de homologação (main 18c345b). Rotina, retenção e observabilidade do ambiente real pendentes.</x:v>
       </x:c>
       <x:c r="E61" s="23" t="str">
         <x:v>A definir</x:v>
@@ -1523,7 +1523,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D62" s="24" t="str">
-        <x:v>Regressões automatizadas foram executadas. UAT e homologação ainda não ocorreram.</x:v>
+        <x:v>Regressões automatizadas e homologação ensaiada com 82 verificações OK (18/10/2026) em main. Roteiro de UAT pronto; UAT com STC e SINFRA não ocorreu.</x:v>
       </x:c>
       <x:c r="E62" s="24" t="str">
         <x:v>Sprint 14</x:v>
@@ -1549,7 +1549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ce700d608074e2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8010caae41974209"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1716,7 +1716,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02cd1a5700b24d46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2f44f52801c4e84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1883,7 +1883,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d7291a4f1b24db1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff7dcd07c46142f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2070,7 +2070,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R807740a09a334e54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa8a6fac238b4ae8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2277,7 +2277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99f9af4a6b1f4826"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re91b783551df4f7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2464,7 +2464,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb30e8e7210bc4038"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568885a3ee15470f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2582,7 +2582,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>O caminho /v1 usa API real. Retirada dos dados demo para homologação permanece pendente.</x:v>
+        <x:v>O caminho /v1 usa API real e, em produção, a imagem serve só a V1. Carga do piloto preparada, mas não executada em base operacional.</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>O caminho variável não depende de dados demonstrativos.</x:v>
@@ -2602,7 +2602,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>O caminho /v1 usa API real. Retirada dos dados demo para homologação permanece pendente.</x:v>
+        <x:v>O caminho /v1 usa API real e, em produção, a imagem serve só a V1. Carga do piloto preparada, mas não executada em base operacional.</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:v>O caminho fixo não depende de dados demonstrativos.</x:v>
@@ -2622,7 +2622,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
-        <x:v>Regressões automatizadas e docker compose build app passaram. UAT e homologação continuam pendentes.</x:v>
+        <x:v>Auditoria e homologação ensaiada sem defeito bloqueante em main (18c345b, PR #11). UAT com STC e SINFRA pendente.</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
         <x:v>Não há defeito bloqueante nos dois fluxos mínimos.</x:v>
@@ -2631,7 +2631,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc60319396364ee8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab957d4a7a341bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(planejamento): alinhar o backlog ao estado da V1
- status e evidências conferidos contra a main de 19/10: fundação
  concluída, adjuntas e texto para o SEI pendentes, PR #13 aberto
- critérios das Sprints 9 e 10 reescritos como critérios verificáveis
- tabelas do Excel alinhadas aos cabeçalhos; a versão anterior só
  abria em modo de reparo
- linhas de dados sem altura fixa, para mostrar o texto inteiro
</commit_message>
<xml_diff>
--- a/planejamento/backlog-completo.xlsx
+++ b/planejamento/backlog-completo.xlsx
@@ -211,8 +211,8 @@
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Atividade macro"/>
     <x:tableColumn id="2" name="Descrição simples"/>
-    <x:tableColumn id="3" name="Parecer Guilherme"/>
-    <x:tableColumn id="4" name="Observações"/>
+    <x:tableColumn id="3" name="Status técnico"/>
+    <x:tableColumn id="4" name="Integração/evidência"/>
     <x:tableColumn id="5" name="Tratamento do plano"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -220,84 +220,90 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Sprint9Table" displayName="Sprint9Table" ref="A4:E8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E8"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Sprint9Table" displayName="Sprint9Table" ref="A4:F9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F9"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Atividade"/>
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
-    <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="4" name="Status técnico"/>
+    <x:tableColumn id="5" name="Integração/evidência"/>
+    <x:tableColumn id="6" name="Critério de aceite"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Sprint10Table" displayName="Sprint10Table" ref="A4:E9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E9"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Sprint10Table" displayName="Sprint10Table" ref="A4:F9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F9"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Atividade"/>
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
-    <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="4" name="Status técnico"/>
+    <x:tableColumn id="5" name="Integração/evidência"/>
+    <x:tableColumn id="6" name="Critério de aceite"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Sprint11Table" displayName="Sprint11Table" ref="A4:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E10"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Sprint11Table" displayName="Sprint11Table" ref="A4:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F10"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Atividade"/>
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
-    <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="4" name="Status técnico"/>
+    <x:tableColumn id="5" name="Integração/evidência"/>
+    <x:tableColumn id="6" name="Critério de aceite"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Sprint12Table" displayName="Sprint12Table" ref="A4:E11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E11"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Sprint12Table" displayName="Sprint12Table" ref="A4:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F11"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Atividade"/>
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
-    <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="4" name="Status técnico"/>
+    <x:tableColumn id="5" name="Integração/evidência"/>
+    <x:tableColumn id="6" name="Critério de aceite"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Sprint13Table" displayName="Sprint13Table" ref="A4:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E10"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Sprint13Table" displayName="Sprint13Table" ref="A4:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F10"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Atividade"/>
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
-    <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="4" name="Status técnico"/>
+    <x:tableColumn id="5" name="Integração/evidência"/>
+    <x:tableColumn id="6" name="Critério de aceite"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Sprint14Table" displayName="Sprint14Table" ref="A4:E9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:E9"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Sprint14Table" displayName="Sprint14Table" ref="A4:F9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F9"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Atividade"/>
     <x:tableColumn id="2" name="Objetivo / entrega"/>
     <x:tableColumn id="3" name="Atividade macro de origem"/>
-    <x:tableColumn id="4" name="Status"/>
-    <x:tableColumn id="5" name="Status"/>
+    <x:tableColumn id="4" name="Status técnico"/>
+    <x:tableColumn id="5" name="Integração/evidência"/>
+    <x:tableColumn id="6" name="Critério de aceite"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -543,7 +549,7 @@
         <x:v>Tratamento do plano</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" hidden="0">
       <x:c r="A5" s="19" t="str">
         <x:v>Consolidar fontes e decisões vigentes da V1</x:v>
       </x:c>
@@ -554,13 +560,13 @@
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
-        <x:v>Governança reconciliada neste snapshot de 12/10/2026.</x:v>
+        <x:v>Governança reconciliada até o PR #12, em 19/10/2026.</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" hidden="0">
       <x:c r="A6" s="20" t="str">
         <x:v>Criar backlog normativo e planilha operacional por sprint</x:v>
       </x:c>
@@ -571,13 +577,13 @@
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
-        <x:v>Governança reconciliada neste snapshot de 12/10/2026.</x:v>
+        <x:v>Governança reconciliada até o PR #12, em 19/10/2026.</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" hidden="0">
       <x:c r="A7" s="20" t="str">
         <x:v>Aplicar os três handoffs de 31/08 somente no snapshot</x:v>
       </x:c>
@@ -588,13 +594,13 @@
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="D7" s="20" t="str">
-        <x:v>Protótipo entregue em agiliza-transparencia/origin/main (5a19a61).</x:v>
+        <x:v>Protótipo entregue no repositório privado EnzoFrazao/agiliza-transparencia (main, 5a19a61).</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+    <x:row r="8" hidden="0">
       <x:c r="A8" s="20" t="str">
         <x:v>Validar visualmente os handoffs em 375, 768, 1024 e 1440 px</x:v>
       </x:c>
@@ -605,13 +611,13 @@
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="D8" s="20" t="str">
-        <x:v>Protótipo entregue em agiliza-transparencia/origin/main (5a19a61).</x:v>
+        <x:v>Protótipo entregue no repositório privado EnzoFrazao/agiliza-transparencia (main, 5a19a61).</x:v>
       </x:c>
       <x:c r="E8" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" hidden="0">
       <x:c r="A9" s="20" t="str">
         <x:v>Reconciliar o backlog com decisões e telas aprovadas</x:v>
       </x:c>
@@ -622,13 +628,13 @@
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="D9" s="20" t="str">
-        <x:v>Backlog e documentos derivados reconciliados neste snapshot de 12/10/2026.</x:v>
+        <x:v>Backlog e documentos derivados reconciliados com o estado da V1 em 19/10/2026.</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="48" hidden="0" customHeight="1">
+    <x:row r="10" hidden="0">
       <x:c r="A10" s="24" t="str">
         <x:v>Inventariar e preparar a migração do ambiente local: interface, API, banco e ferramentas</x:v>
       </x:c>
@@ -645,7 +651,7 @@
         <x:v>Sprint 9</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="72" hidden="0" customHeight="1">
+    <x:row r="11" hidden="0">
       <x:c r="A11" s="24" t="str">
         <x:v>Consolidar no repositório canônico guia, backlog, contratos-alvo e specs sanitizadas</x:v>
       </x:c>
@@ -662,7 +668,7 @@
         <x:v>Sprint 9</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="60" hidden="0" customHeight="1">
+    <x:row r="12" hidden="0">
       <x:c r="A12" s="24" t="str">
         <x:v>Migrar seletivamente interface e API ao repositório canônico e ao único container de aplicação</x:v>
       </x:c>
@@ -673,13 +679,13 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Interface e API da V1 em main (60f25d0, PR #5 mesclado em 14/10/2026); em produção a imagem serve só a V1 (18c345b). Falta retirar os dados demonstrativos do protótipo (Sprint 14).</x:v>
       </x:c>
       <x:c r="E12" s="24" t="str">
         <x:v>Sprint 9 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="72" hidden="0" customHeight="1">
+    <x:row r="13" hidden="0">
       <x:c r="A13" s="24" t="str">
         <x:v>Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
@@ -687,16 +693,16 @@
         <x:v>Prepara a aplicação Laravel, o PostgreSQL externo e o desenvolvimento no container único.</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
+        <x:v>Laravel com PostgreSQL externo no Compose de desenvolvimento, em main. Migrations de ida e volta e suíte em PostgreSQL 17 passaram em 19/10/2026. O PostgreSQL institucional segue com a fundação de homologação.</x:v>
       </x:c>
       <x:c r="E13" s="24" t="str">
         <x:v>Sprint 9 e Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="48" hidden="0" customHeight="1">
+    <x:row r="14" hidden="0">
       <x:c r="A14" s="20" t="str">
         <x:v>Implementar health check, logs básicos e gate unificado de testes da aplicação</x:v>
       </x:c>
@@ -713,7 +719,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+    <x:row r="15" hidden="0">
       <x:c r="A15" s="24" t="str">
         <x:v>Definir contexto de ator controlado e autorização desacoplada do login</x:v>
       </x:c>
@@ -730,7 +736,7 @@
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="60" hidden="0" customHeight="1">
+    <x:row r="16" hidden="0">
       <x:c r="A16" s="24" t="str">
         <x:v>Aprovar e implementar o primeiro contrato HTTP real e cliente TypeScript</x:v>
       </x:c>
@@ -747,7 +753,7 @@
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
+    <x:row r="17" hidden="0">
       <x:c r="A17" s="20" t="str">
         <x:v>Preparar fundação de homologação da aplicação em container único</x:v>
       </x:c>
@@ -758,13 +764,13 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D17" s="20" t="str">
-        <x:v>Imagem de produção ensaiada atrás de proxy HTTPS, com guia do ambiente e roteiro de UAT, em main (18c345b, PR #11 mesclado em 19/10/2026). Ambiente real e hospedagem pendentes.</x:v>
+        <x:v>Imagem de produção ensaiada atrás de proxy HTTPS, com guia do ambiente e roteiro de UAT, em main (18c345b, PR #11 mesclado em 19/10/2026). A correção dos processos PHP da imagem está no PR #13, aberto. Ambiente real e hospedagem pendentes.</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+    <x:row r="18" hidden="0">
       <x:c r="A18" s="24" t="str">
         <x:v>Persistir o Catálogo mínimo e as UGs necessárias à publicação</x:v>
       </x:c>
@@ -781,7 +787,7 @@
         <x:v>Sprint 11 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
+    <x:row r="19" hidden="0">
       <x:c r="A19" s="24" t="str">
         <x:v>Configurar ciclo de objeto variável sem modelo XLSX obrigatório</x:v>
       </x:c>
@@ -792,13 +798,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 18/10/2026 o variável é configurado no ato, com lista de informações solicitadas e sem objeto do Catálogo (main 18c345b).</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
         <x:v>Sprint 11</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+    <x:row r="20" hidden="0">
       <x:c r="A20" s="24" t="str">
         <x:v>Cadastrar e versionar modelo XLSX oficial obrigatório por objeto fixo</x:v>
       </x:c>
@@ -815,7 +821,7 @@
         <x:v>Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
+    <x:row r="21" hidden="0">
       <x:c r="A21" s="24" t="str">
         <x:v>Publicar ciclo de modo atômico e idempotente</x:v>
       </x:c>
@@ -832,7 +838,7 @@
         <x:v>Sprint 11 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
+    <x:row r="22" hidden="0">
       <x:c r="A22" s="20" t="str">
         <x:v>Publicar sem SEI e congelar toggle focal por UG</x:v>
       </x:c>
@@ -849,7 +855,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
+    <x:row r="23" hidden="0">
       <x:c r="A23" s="24" t="str">
         <x:v>Integrar Criar Ciclo, Ciclos e Detalhe ao backend</x:v>
       </x:c>
@@ -866,7 +872,7 @@
         <x:v>Sprint 11 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
+    <x:row r="24" hidden="0">
       <x:c r="A24" s="20" t="str">
         <x:v>Auditar criação e publicação do ciclo</x:v>
       </x:c>
@@ -877,13 +883,13 @@
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="D24" s="20" t="str">
-        <x:v>Não iniciado no repositório canônico.</x:v>
+        <x:v>O ciclo guarda quem o criou; não há trilha de auditoria da criação e da publicação.</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
+    <x:row r="25" hidden="0">
       <x:c r="A25" s="20" t="str">
         <x:v>Convidar respondentes e adjuntas por e-mail institucional</x:v>
       </x:c>
@@ -900,7 +906,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
+    <x:row r="26" hidden="0">
       <x:c r="A26" s="24" t="str">
         <x:v>Criar atribuição e contribuição separada por pessoa e adjunta</x:v>
       </x:c>
@@ -908,16 +914,16 @@
         <x:v>Define a atribuição de cada pessoa e separa a contribuição da adjunta.</x:v>
       </x:c>
       <x:c r="C26" s="24" t="str">
-        <x:v>Concluído tecnicamente</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Acesso e rascunho por pessoa em main (60f25d0, PR #5 mesclado em 14/10/2026). Adjuntas não implementadas. Desde 18/10/2026 cada UG envia uma única resposta (main 18c345b).</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
         <x:v>Sprint 12</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
+    <x:row r="27" hidden="0">
       <x:c r="A27" s="24" t="str">
         <x:v>Receber campos diretos e uploads em objeto variável sem modelo XLSX obrigatório</x:v>
       </x:c>
@@ -934,7 +940,7 @@
         <x:v>Sprint 12</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
+    <x:row r="28" hidden="0">
       <x:c r="A28" s="24" t="str">
         <x:v>Baixar, preencher e enviar o modelo XLSX oficial obrigatório do objeto fixo</x:v>
       </x:c>
@@ -951,7 +957,7 @@
         <x:v>Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
+    <x:row r="29" hidden="0">
       <x:c r="A29" s="24" t="str">
         <x:v>Salvar rascunho e arquivos vigentes em storage desacoplado</x:v>
       </x:c>
@@ -968,7 +974,7 @@
         <x:v>Sprint 12 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
+    <x:row r="30" hidden="0">
       <x:c r="A30" s="24" t="str">
         <x:v>Enviar pacote completo e emitir comprovante auditável</x:v>
       </x:c>
@@ -985,7 +991,7 @@
         <x:v>Sprint 12 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
+    <x:row r="31" hidden="0">
       <x:c r="A31" s="24" t="str">
         <x:v>Integrar painéis e contribuição às APIs da sprint</x:v>
       </x:c>
@@ -1002,7 +1008,7 @@
         <x:v>Sprint 12 e Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
+    <x:row r="32" hidden="0">
       <x:c r="A32" s="20" t="str">
         <x:v>Aplicar modos direto, focal coordenador e focal observador</x:v>
       </x:c>
@@ -1019,7 +1025,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
+    <x:row r="33" hidden="0">
       <x:c r="A33" s="20" t="str">
         <x:v>Preservar o escopo durante a revisão focal</x:v>
       </x:c>
@@ -1036,7 +1042,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
+    <x:row r="34" hidden="0">
       <x:c r="A34" s="20" t="str">
         <x:v>Declarar ausência total de informações</x:v>
       </x:c>
@@ -1053,7 +1059,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
+    <x:row r="35" hidden="0">
       <x:c r="A35" s="24" t="str">
         <x:v>Detectar campo direto ou upload ausente em objeto variável antes do envio</x:v>
       </x:c>
@@ -1070,7 +1076,7 @@
         <x:v>Sprint 11 e Sprint 12</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="15" hidden="0" customHeight="1">
+    <x:row r="36" hidden="0">
       <x:c r="A36" s="24" t="str">
         <x:v>Validar o modelo XLSX obrigatório do objeto fixo antes do envio</x:v>
       </x:c>
@@ -1087,7 +1093,7 @@
         <x:v>Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="15" hidden="0" customHeight="1">
+    <x:row r="37" hidden="0">
       <x:c r="A37" s="20" t="str">
         <x:v>Confirmar não ocorrências e manter resposta parcial como respondida</x:v>
       </x:c>
@@ -1104,7 +1110,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="15" hidden="0" customHeight="1">
+    <x:row r="38" hidden="0">
       <x:c r="A38" s="20" t="str">
         <x:v>Conferir contribuições e encaminhar o conjunto focal à STC</x:v>
       </x:c>
@@ -1121,7 +1127,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="15" hidden="0" customHeight="1">
+    <x:row r="39" hidden="0">
       <x:c r="A39" s="20" t="str">
         <x:v>Apresentar pacote e completude para decisão humana da STC</x:v>
       </x:c>
@@ -1138,7 +1144,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="15" hidden="0" customHeight="1">
+    <x:row r="40" hidden="0">
       <x:c r="A40" s="20" t="str">
         <x:v>Devolver contribuição ou item específico com um motivo</x:v>
       </x:c>
@@ -1155,7 +1161,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="15" hidden="0" customHeight="1">
+    <x:row r="41" hidden="0">
       <x:c r="A41" s="20" t="str">
         <x:v>Corrigir e reenviar somente a contribuição afetada</x:v>
       </x:c>
@@ -1172,7 +1178,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="15" hidden="0" customHeight="1">
+    <x:row r="42" hidden="0">
       <x:c r="A42" s="20" t="str">
         <x:v>Persistir o estado do ciclo, validar e permitir reversão controlada</x:v>
       </x:c>
@@ -1189,7 +1195,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="15" hidden="0" customHeight="1">
+    <x:row r="43" hidden="0">
       <x:c r="A43" s="20" t="str">
         <x:v>Separar auditoria de ciclo, coleta e respostas</x:v>
       </x:c>
@@ -1206,7 +1212,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="15" hidden="0" customHeight="1">
+    <x:row r="44" hidden="0">
       <x:c r="A44" s="20" t="str">
         <x:v>Integrar Validação e Histórico às APIs reais</x:v>
       </x:c>
@@ -1223,7 +1229,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="15" hidden="0" customHeight="1">
+    <x:row r="45" hidden="0">
       <x:c r="A45" s="20" t="str">
         <x:v>Registrar números SEI e iniciar ou reiterar o prazo</x:v>
       </x:c>
@@ -1240,7 +1246,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="15" hidden="0" customHeight="1">
+    <x:row r="46" hidden="0">
       <x:c r="A46" s="20" t="str">
         <x:v>Operar duas prorrogações separadas de cinco dias úteis</x:v>
       </x:c>
@@ -1257,7 +1263,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="15" hidden="0" customHeight="1">
+    <x:row r="47" hidden="0">
       <x:c r="A47" s="20" t="str">
         <x:v>Tratar solicitações de prorrogação pelo modo da UG</x:v>
       </x:c>
@@ -1274,7 +1280,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" ht="15" hidden="0" customHeight="1">
+    <x:row r="48" hidden="0">
       <x:c r="A48" s="20" t="str">
         <x:v>Encerrar manualmente coleta e ciclo</x:v>
       </x:c>
@@ -1291,7 +1297,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="15" hidden="0" customHeight="1">
+    <x:row r="49" hidden="0">
       <x:c r="A49" s="20" t="str">
         <x:v>Manter e exportar o Catálogo para ciclos futuros</x:v>
       </x:c>
@@ -1308,7 +1314,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="15" hidden="0" customHeight="1">
+    <x:row r="50" hidden="0">
       <x:c r="A50" s="20" t="str">
         <x:v>Entregar dashboard operacional com unidades e drill-downs explícitos</x:v>
       </x:c>
@@ -1325,7 +1331,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="15" hidden="0" customHeight="1">
+    <x:row r="51" hidden="0">
       <x:c r="A51" s="20" t="str">
         <x:v>Completar Histórico e consultas do Gabinete</x:v>
       </x:c>
@@ -1342,7 +1348,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="15" hidden="0" customHeight="1">
+    <x:row r="52" hidden="0">
       <x:c r="A52" s="20" t="str">
         <x:v>Copiar link e texto manual para uso no processo SEI</x:v>
       </x:c>
@@ -1350,16 +1356,16 @@
         <x:v>Gera link e texto para copiar manualmente no processo SEI.</x:v>
       </x:c>
       <x:c r="C52" s="20" t="str">
-        <x:v>Planejado</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D52" s="20" t="str">
-        <x:v>Não iniciado no repositório canônico.</x:v>
+        <x:v>Copiar link e Girar link em main (18c345b, PR #11). Texto para o processo SEI não implementado.</x:v>
       </x:c>
       <x:c r="E52" s="23" t="str">
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" ht="15" hidden="0" customHeight="1">
+    <x:row r="53" hidden="0">
       <x:c r="A53" s="20" t="str">
         <x:v>Operar o Diretório de UGs como consulta contextual</x:v>
       </x:c>
@@ -1376,7 +1382,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="15" hidden="0" customHeight="1">
+    <x:row r="54" hidden="0">
       <x:c r="A54" s="20" t="str">
         <x:v>Excluir ciclo sem apagar respostas armazenadas</x:v>
       </x:c>
@@ -1393,7 +1399,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" ht="15" hidden="0" customHeight="1">
+    <x:row r="55" hidden="0">
       <x:c r="A55" s="24" t="str">
         <x:v>Conectar login institucional ao contexto de ator</x:v>
       </x:c>
@@ -1410,7 +1416,7 @@
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="15" hidden="0" customHeight="1">
+    <x:row r="56" hidden="0">
       <x:c r="A56" s="24" t="str">
         <x:v>Conectar acesso contextual pelo link estável</x:v>
       </x:c>
@@ -1427,7 +1433,7 @@
         <x:v>Sprint 11 e Sprint 12 e Sprint 13</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="15" hidden="0" customHeight="1">
+    <x:row r="57" hidden="0">
       <x:c r="A57" s="24" t="str">
         <x:v>Aplicar isolamento definitivo de perfis, UGs e capacidades</x:v>
       </x:c>
@@ -1444,7 +1450,7 @@
         <x:v>Sprint 10</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" ht="15" hidden="0" customHeight="1">
+    <x:row r="58" hidden="0">
       <x:c r="A58" s="20" t="str">
         <x:v>Exportar o filtro atual do Histórico em XLSX macro</x:v>
       </x:c>
@@ -1461,7 +1467,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" ht="15" hidden="0" customHeight="1">
+    <x:row r="59" hidden="0">
       <x:c r="A59" s="24" t="str">
         <x:v>Remover dados fictícios e acessos de demonstração do build de homologação</x:v>
       </x:c>
@@ -1478,7 +1484,7 @@
         <x:v>Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="15" hidden="0" customHeight="1">
+    <x:row r="60" hidden="0">
       <x:c r="A60" s="20" t="str">
         <x:v>Fechar segurança, upload, privacidade e retenção mínimas para o piloto</x:v>
       </x:c>
@@ -1495,7 +1501,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="15" hidden="0" customHeight="1">
+    <x:row r="61" hidden="0">
       <x:c r="A61" s="20" t="str">
         <x:v>Verificar observabilidade, backup, recuperação e rollback em homologação</x:v>
       </x:c>
@@ -1512,7 +1518,7 @@
         <x:v>A definir</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" ht="15" hidden="0" customHeight="1">
+    <x:row r="62" hidden="0">
       <x:c r="A62" s="24" t="str">
         <x:v>Executar acessibilidade, responsividade, regressão e UAT ponta a ponta</x:v>
       </x:c>
@@ -1523,13 +1529,13 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D62" s="24" t="str">
-        <x:v>Regressões automatizadas e homologação ensaiada com 82 verificações OK (18/10/2026) em main. Roteiro de UAT pronto; UAT com STC e SINFRA não ocorreu.</x:v>
+        <x:v>Regressões automatizadas e homologação ensaiada com 82 verificações OK (18/10/2026) em main. Roteiro de UAT pronto; UAT com STC e SINFRA não ocorreu. Adiantamento: como a V1 está à frente das Sprints 12–14, ela será apresentada à chefia em 20/10/2026 e aberta para teste de usabilidade. Os ajustes e o uso pela SINFRA ainda não têm data.</x:v>
       </x:c>
       <x:c r="E62" s="24" t="str">
         <x:v>Sprint 14</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" ht="15" hidden="0" customHeight="1">
+    <x:row r="63" hidden="0">
       <x:c r="A63" s="21" t="str">
         <x:v>Emitir decisão de prontidão para piloto em homologação</x:v>
       </x:c>
@@ -1540,7 +1546,7 @@
         <x:v>Planejado</x:v>
       </x:c>
       <x:c r="D63" s="21" t="str">
-        <x:v>Não iniciado no repositório canônico.</x:v>
+        <x:v>Não emitida. Os ajustes pedidos pela chefia no teste de usabilidade devem anteceder o uso pela SINFRA.</x:v>
       </x:c>
       <x:c r="E63" s="25" t="str">
         <x:v>A definir</x:v>
@@ -1613,7 +1619,7 @@
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="24" hidden="0" customHeight="1">
+    <x:row r="5" hidden="0">
       <x:c r="A5" s="19" t="str">
         <x:v>Inventariar código, banco e ferramentas</x:v>
       </x:c>
@@ -1633,7 +1639,7 @@
         <x:v>Inventário, fluxo e regras foram preparados para revisão técnica.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" hidden="0" customHeight="1">
+    <x:row r="6" hidden="0">
       <x:c r="A6" s="20" t="str">
         <x:v>Preparar o repositório canônico</x:v>
       </x:c>
@@ -1647,13 +1653,13 @@
         <x:v>Concluído</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
-        <x:v>Repositório canônico criado. Integração técnica segue em main e na branch V1.</x:v>
+        <x:v>Repositório canônico criado; interface e API da V1 integradas em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
-        <x:v>Repositório canônico criado; a migração seletiva do frontend foi implementada em fix-migracao e aguarda PR/merge.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>O repositório canônico existe e o pacote de transporte entra nele só depois de URL e branch informadas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" hidden="0">
       <x:c r="A7" s="20" t="str">
         <x:v>Iniciar o container único</x:v>
       </x:c>
@@ -1664,16 +1670,16 @@
         <x:v>Inventariar e preparar a migração do ambiente local: interface, API, banco e ferramentas | Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
       <x:c r="D7" s="29" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
+        <x:v>Container da aplicação separado do PostgreSQL no Compose de desenvolvimento; docker compose build app verificado em 14/10/2026 e imagem de produção ensaiada (main 18c345b).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
-        <x:v>Não há container de aplicação configurado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="24" hidden="0" customHeight="1">
+        <x:v>O container da aplicação sobe separado do container PostgreSQL de desenvolvimento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" hidden="0">
       <x:c r="A8" s="21" t="str">
         <x:v>Iniciar Laravel e a conexão PostgreSQL</x:v>
       </x:c>
@@ -1684,16 +1690,16 @@
         <x:v>Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E8" s="31" t="str">
-        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
+        <x:v>Laravel/Inertia conectado ao PostgreSQL externo por variáveis de ambiente; migrations e suíte em PostgreSQL 17 passaram em 19/10/2026. O PostgreSQL institucional segue com a fundação de homologação.</x:v>
       </x:c>
       <x:c r="F8" s="21" t="str">
-        <x:v>Laravel/Inertia existe; PostgreSQL externo ainda não foi configurado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>O Laravel lê a conexão PostgreSQL por variáveis de ambiente e roda as migrations no container de desenvolvimento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" hidden="0">
       <x:c r="A9" s="35" t="str">
         <x:v>Preparar fluxo e regras do backend</x:v>
       </x:c>
@@ -1707,10 +1713,10 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="35" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Fluxo, regras e handoff em documentos/governanca; o fluxo foi implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F9" s="35" t="str">
-        <x:v>Fluxo V1, regras e handoff técnico documentados; contrato HTTP continua pendente.</x:v>
+        <x:v>Fluxo V1, regras de validação, estados e critérios de aceite documentados para a revisão técnica.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1780,7 +1786,7 @@
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="24" hidden="0" customHeight="1">
+    <x:row r="5" hidden="0">
       <x:c r="A5" s="19" t="str">
         <x:v>Concluir a fundação Laravel e PostgreSQL</x:v>
       </x:c>
@@ -1791,16 +1797,16 @@
         <x:v>Criar fundação Laravel com PostgreSQL externo e configuração de desenvolvimento compatível com o container único</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Em andamento</x:v>
+        <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Base em main (60f25d0). PostgreSQL e migrations validados; docker compose build app verificado em 14/10/2026.</x:v>
+        <x:v>Migrations mínimas, configuração local e execução com PostgreSQL externo em main; suíte em PostgreSQL 17 com migrations de ida e volta em 19/10/2026.</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
-        <x:v>Laravel/Inertia iniciado; PostgreSQL externo bloqueado até alinhamento técnico com a STC.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="24" hidden="0" customHeight="1">
+        <x:v>A aplicação roda com as migrations mínimas aplicadas no PostgreSQL externo de desenvolvimento.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" hidden="0">
       <x:c r="A6" s="20" t="str">
         <x:v>Criar o primeiro endpoint HTTP</x:v>
       </x:c>
@@ -1817,10 +1823,10 @@
         <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
-        <x:v>Aguardar contrato de dados, infraestrutura e estratégia de homologação definidos com a STC.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>Uma rota de API real responde a partir do backend Laravel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" hidden="0">
       <x:c r="A7" s="20" t="str">
         <x:v>Conectar a primeira tela à API</x:v>
       </x:c>
@@ -1837,10 +1843,10 @@
         <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
-        <x:v>Depende do primeiro contrato HTTP aprovado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="24" hidden="0" customHeight="1">
+        <x:v>Uma tela consome a rota real pelo cliente TypeScript, sem dados demonstrativos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" hidden="0">
       <x:c r="A8" s="20" t="str">
         <x:v>Criar grupos Administrador/STC e Respondente</x:v>
       </x:c>
@@ -1860,7 +1866,7 @@
         <x:v>Administrador/STC e Respondente possuem ações diferentes no MVP.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" hidden="0">
       <x:c r="A9" s="21" t="str">
         <x:v>Vincular usuários a UGs e grupos</x:v>
       </x:c>
@@ -1947,7 +1953,7 @@
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="44" customHeight="1">
+    <x:row r="5">
       <x:c r="A5" s="19" t="str">
         <x:v>Carregar um objeto variável e uma UG</x:v>
       </x:c>
@@ -1961,13 +1967,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 18/10/2026 o variável é configurado no ato, sem objeto do Catálogo, e o MT-0018 fixo tem carga controlada preparada (main 18c345b).</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>STC seleciona um objeto variável e uma UG.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+    <x:row r="6">
       <x:c r="A6" s="20" t="str">
         <x:v>Criar o formulário da coleta variável</x:v>
       </x:c>
@@ -1981,13 +1987,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E6" s="29" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 18/10/2026 com lista de informações solicitadas (main 18c345b).</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
         <x:v>STC cria uma coleta variável com objeto, UG e item solicitado.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="60" customHeight="1">
+    <x:row r="7">
       <x:c r="A7" s="20" t="str">
         <x:v>Definir upload obrigatório no objeto variável</x:v>
       </x:c>
@@ -2007,7 +2013,7 @@
         <x:v>A coleta variável deixa explícita a exigência de upload.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+    <x:row r="8">
       <x:c r="A8" s="20" t="str">
         <x:v>Publicar a coleta variável</x:v>
       </x:c>
@@ -2027,7 +2033,7 @@
         <x:v>A publicação cria uma coleta sem estado parcial.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+    <x:row r="9">
       <x:c r="A9" s="20" t="str">
         <x:v>Gerar link único da coleta</x:v>
       </x:c>
@@ -2047,7 +2053,7 @@
         <x:v>Abrir o link leva ao pedido correspondente.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="44" customHeight="1">
+    <x:row r="10">
       <x:c r="A10" s="21" t="str">
         <x:v>Conectar criação, lista e detalhe da STC</x:v>
       </x:c>
@@ -2134,7 +2140,7 @@
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="44" customHeight="1">
+    <x:row r="5">
       <x:c r="A5" s="19" t="str">
         <x:v>Abrir acesso público pelo link</x:v>
       </x:c>
@@ -2154,7 +2160,7 @@
         <x:v>O link não mostra pedidos de outras UGs.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+    <x:row r="6">
       <x:c r="A6" s="20" t="str">
         <x:v>Identificar o respondente no acesso inicial</x:v>
       </x:c>
@@ -2174,7 +2180,7 @@
         <x:v>O respondente entra na contribuição correta sem SSO institucional completo.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+    <x:row r="7">
       <x:c r="A7" s="20" t="str">
         <x:v>Exibir campos e anexos do objeto variável</x:v>
       </x:c>
@@ -2188,13 +2194,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E7" s="29" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 17/10/2026 a resposta é só por arquivos, sem campos diretos (main 18c345b).</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
         <x:v>O respondente visualiza os itens solicitados.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="60" customHeight="1">
+    <x:row r="8">
       <x:c r="A8" s="20" t="str">
         <x:v>Guardar o upload variável até o envio</x:v>
       </x:c>
@@ -2208,13 +2214,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 17/10/2026 o arquivo fica guardado ao ser escolhido, sem Salvar rascunho (main 18c345b).</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
         <x:v>O arquivo permanece disponível até o envio da resposta.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+    <x:row r="9">
       <x:c r="A9" s="20" t="str">
         <x:v>Bloquear envio variável sem arquivo</x:v>
       </x:c>
@@ -2228,13 +2234,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E9" s="29" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Desde 17/10/2026 não há campos diretos; o envio exige ao menos um arquivo (main 18c345b).</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
         <x:v>O sistema bloqueia o envio quando não existe upload.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="44" customHeight="1">
+    <x:row r="10">
       <x:c r="A10" s="20" t="str">
         <x:v>Enviar a resposta variável</x:v>
       </x:c>
@@ -2248,13 +2254,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E10" s="24" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Comprovante PDF desde o PR #10 (16/10/2026); desde 18/10/2026 cada UG envia uma única resposta (main 18c345b).</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
         <x:v>A resposta sai do respondente e fica disponível para a STC.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="44" customHeight="1">
+    <x:row r="11">
       <x:c r="A11" s="21" t="str">
         <x:v>Exibir e baixar a resposta variável na STC</x:v>
       </x:c>
@@ -2341,7 +2347,7 @@
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="60" customHeight="1">
+    <x:row r="5">
       <x:c r="A5" s="19" t="str">
         <x:v>Cadastrar um objeto fixo</x:v>
       </x:c>
@@ -2355,13 +2361,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Na V1, o MT-0018 entra por carga controlada (catalog:load-pilot), sem cadastro pela STC; a carga operacional não foi executada.</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>Existe um objeto fixo disponível para criar uma coleta.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+    <x:row r="6">
       <x:c r="A6" s="20" t="str">
         <x:v>Associar um único XLSX oficial</x:v>
       </x:c>
@@ -2381,7 +2387,7 @@
         <x:v>O objeto fixo possui um modelo XLSX disponível.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="44" customHeight="1">
+    <x:row r="7">
       <x:c r="A7" s="20" t="str">
         <x:v>Criar e publicar a coleta fixa</x:v>
       </x:c>
@@ -2401,7 +2407,7 @@
         <x:v>A coleta fixa tem link próprio e referência ao modelo.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+    <x:row r="8">
       <x:c r="A8" s="20" t="str">
         <x:v>Disponibilizar download do XLSX oficial</x:v>
       </x:c>
@@ -2421,7 +2427,7 @@
         <x:v>O respondente baixa o XLSX vinculado à coleta fixa.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="60" customHeight="1">
+    <x:row r="9">
       <x:c r="A9" s="20" t="str">
         <x:v>Receber o XLSX preenchido</x:v>
       </x:c>
@@ -2441,7 +2447,7 @@
         <x:v>O respondente envia a planilha preenchida como arquivo principal.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="44" customHeight="1">
+    <x:row r="10">
       <x:c r="A10" s="21" t="str">
         <x:v>Conferir o XLSX mínimo</x:v>
       </x:c>
@@ -2528,7 +2534,7 @@
         <x:v>Critério de aceite</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="44" customHeight="1">
+    <x:row r="5">
       <x:c r="A5" s="19" t="str">
         <x:v>Enviar a resposta fixa</x:v>
       </x:c>
@@ -2542,13 +2548,13 @@
         <x:v>Concluído tecnicamente</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
-        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026).</x:v>
+        <x:v>Implementado em main (60f25d0, PR #5 mesclado em 14/10/2026). Comprovante PDF em main (849c522, PR #10 mesclado em 16/10/2026).</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>A resposta fixa fica disponível para a STC.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="44" customHeight="1">
+    <x:row r="6">
       <x:c r="A6" s="20" t="str">
         <x:v>Exibir e baixar a resposta fixa na STC</x:v>
       </x:c>
@@ -2568,7 +2574,7 @@
         <x:v>STC localiza e baixa a planilha oficial.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="76" customHeight="1">
+    <x:row r="7">
       <x:c r="A7" s="20" t="str">
         <x:v>Retirar dados demo do caminho variável</x:v>
       </x:c>
@@ -2588,7 +2594,7 @@
         <x:v>O caminho variável não depende de dados demonstrativos.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="76" customHeight="1">
+    <x:row r="8">
       <x:c r="A8" s="20" t="str">
         <x:v>Retirar dados demo do caminho fixo</x:v>
       </x:c>
@@ -2608,7 +2614,7 @@
         <x:v>O caminho fixo não depende de dados demonstrativos.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="44" customHeight="1">
+    <x:row r="9">
       <x:c r="A9" s="21" t="str">
         <x:v>Corrigir defeitos bloqueantes</x:v>
       </x:c>
@@ -2622,7 +2628,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
-        <x:v>Auditoria e homologação ensaiada sem defeito bloqueante em main (18c345b, PR #11). UAT com STC e SINFRA pendente.</x:v>
+        <x:v>Auditoria e homologação ensaiada em main (18c345b, PR #11). A revisão do PR achou depois um bloqueio na imagem (um único processo PHP), corrigido no PR #13, aberto. UAT com STC e SINFRA pendente.</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
         <x:v>Não há defeito bloqueante nos dois fluxos mínimos.</x:v>

</xml_diff>

<commit_message>
docs(planejamento): corrigir a origem de uma atividade da Sprint 9
"Preparar fluxo e regras do backend" apontava para uma atividade
macro inexistente. Passa a apontar para "Consolidar fontes e decisões
vigentes da V1", agora tratada na Sprint 9 também na rastreabilidade.
</commit_message>
<xml_diff>
--- a/planejamento/backlog-completo.xlsx
+++ b/planejamento/backlog-completo.xlsx
@@ -563,7 +563,7 @@
         <x:v>Governança reconciliada até o PR #12, em 19/10/2026.</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
-        <x:v>A definir</x:v>
+        <x:v>Sprint 9</x:v>
       </x:c>
     </x:row>
     <x:row r="6" hidden="0">
@@ -1707,7 +1707,7 @@
         <x:v>Descrever o fluxo MVP fixo/variável, regras de validação, estados e critérios de aceite para revisão de Guilherme.</x:v>
       </x:c>
       <x:c r="C9" s="35" t="str">
-        <x:v>Definir o fluxo principal de coleta, resposta, validação e entrega da V1</x:v>
+        <x:v>Consolidar fontes e decisões vigentes da V1</x:v>
       </x:c>
       <x:c r="D9" s="35" t="str">
         <x:v>Concluído tecnicamente</x:v>

</xml_diff>

<commit_message>
docs(planejamento): registrar o merge do PR #13 no backlog
O PR #13 do agiliza-stc entrou na main em 20/10/2026 (dec25e9). As células
D17 (Lista completa) e E9 (Sprint 14) deixam de dizer que ele está aberto.
Relatório de mudanças e SHA-256 do inventário atualizados.
</commit_message>
<xml_diff>
--- a/planejamento/backlog-completo.xlsx
+++ b/planejamento/backlog-completo.xlsx
@@ -764,7 +764,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="D17" s="20" t="str">
-        <x:v>Imagem de produção ensaiada atrás de proxy HTTPS, com guia do ambiente e roteiro de UAT, em main (18c345b, PR #11 mesclado em 19/10/2026). A correção dos processos PHP da imagem está no PR #13, aberto. Ambiente real e hospedagem pendentes.</x:v>
+        <x:v>Imagem de produção ensaiada atrás de proxy HTTPS, com guia do ambiente e roteiro de UAT, em main (18c345b, PR #11 mesclado em 19/10/2026). A correção dos processos PHP da imagem entrou em main pelo PR #13 (dec25e9, mesclado em 20/10/2026). Ambiente real e hospedagem pendentes.</x:v>
       </x:c>
       <x:c r="E17" s="23" t="str">
         <x:v>A definir</x:v>
@@ -2628,7 +2628,7 @@
         <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="E9" s="32" t="str">
-        <x:v>Auditoria e homologação ensaiada em main (18c345b, PR #11). A revisão do PR achou depois um bloqueio na imagem (um único processo PHP), corrigido no PR #13, aberto. UAT com STC e SINFRA pendente.</x:v>
+        <x:v>Auditoria e homologação ensaiada em main (18c345b, PR #11). A revisão do PR achou depois um bloqueio na imagem (um único processo PHP), corrigido em main pelo PR #13 (dec25e9, mesclado em 20/10/2026). UAT com STC e SINFRA pendente.</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
         <x:v>Não há defeito bloqueante nos dois fluxos mínimos.</x:v>

</xml_diff>